<commit_message>
Entrega 2 Proyecto Optimizador Carteras
</commit_message>
<xml_diff>
--- a/FILES/INPUTS/DICCIONARIO_TICKERS.xlsx
+++ b/FILES/INPUTS/DICCIONARIO_TICKERS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\landa\OneDrive\Escritorio\R_Para_Las_Finanzas_Rodrigo_Escobar\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\landa\OneDrive\Escritorio\R_Para_Las_Finanzas_Rodrigo_Escobar\FILES\INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB7CD232-6B67-485F-9D52-58FFCCE37134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523B2C8D-1666-4B77-8C57-49AC32223625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{C769B749-9B38-4F61-8013-263B4B02318E}"/>
+    <workbookView xWindow="9732" yWindow="2508" windowWidth="8256" windowHeight="8448" xr2:uid="{C769B749-9B38-4F61-8013-263B4B02318E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -4514,7 +4514,7 @@
     <t>LOCAL</t>
   </si>
   <si>
-    <t>EXTANJERA</t>
+    <t>EXTRANJERA</t>
   </si>
 </sst>
 </file>

</xml_diff>